<commit_message>
Upload my Pivot tables excel workbook with patient records
</commit_message>
<xml_diff>
--- a/excel-files/day - 04 Pivottables.xlsx
+++ b/excel-files/day - 04 Pivottables.xlsx
@@ -8,18 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/12a4f0da8943f55f/Data Science Journey/healthcare-analyst-journey/Excel Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{BF008E21-8F15-434A-9573-7B06CB0E69F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BCB0947-4528-45E0-BA96-EF6D095FE014}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{BF008E21-8F15-434A-9573-7B06CB0E69F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45E9580C-B8D0-4905-8B8C-DBEFD08F969A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DFD9C989-F79E-4CE8-B412-25F7762E6C96}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{DFD9C989-F79E-4CE8-B412-25F7762E6C96}"/>
   </bookViews>
   <sheets>
-    <sheet name="Patient_records" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Pivot_reports" sheetId="4" r:id="rId1"/>
+    <sheet name="Department_info" sheetId="3" r:id="rId2"/>
+    <sheet name="Patient_records" sheetId="2" r:id="rId3"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="127">
   <si>
     <t>Yes</t>
   </si>
@@ -340,13 +342,100 @@
   </si>
   <si>
     <t>Patient ID</t>
+  </si>
+  <si>
+    <t>Dr. Reddy</t>
+  </si>
+  <si>
+    <t>D005</t>
+  </si>
+  <si>
+    <t>Dr. Sharma</t>
+  </si>
+  <si>
+    <t>D004</t>
+  </si>
+  <si>
+    <t>Dr. Kumar</t>
+  </si>
+  <si>
+    <t>D003</t>
+  </si>
+  <si>
+    <t>Dr. Mehta</t>
+  </si>
+  <si>
+    <t>D002</t>
+  </si>
+  <si>
+    <t>Dr. Rao</t>
+  </si>
+  <si>
+    <t>D001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bed Occupency </t>
+  </si>
+  <si>
+    <t>Bed occupency %</t>
+  </si>
+  <si>
+    <t>Average Patient Age per department</t>
+  </si>
+  <si>
+    <t>No of Patients per doctor</t>
+  </si>
+  <si>
+    <t>Floor</t>
+  </si>
+  <si>
+    <t>DepartmentID</t>
+  </si>
+  <si>
+    <t>DepartmentName</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>Count of Senior category</t>
+  </si>
+  <si>
+    <t>Departments</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
+    <t>Count of Patient ID</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Months</t>
+  </si>
+  <si>
+    <t>Average of Age</t>
+  </si>
+  <si>
+    <t>(All)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -362,8 +451,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,8 +480,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -385,19 +495,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -410,95 +578,2387 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Patient_Records"/>
-      <sheetName val="Department_info"/>
-      <sheetName val="Pivot_reports"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="2">
-          <cell r="A2" t="str">
-            <v>Cardiology</v>
-          </cell>
-          <cell r="B2" t="str">
-            <v>D001</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>Dr. Rao</v>
-          </cell>
-          <cell r="E2">
-            <v>50</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3" t="str">
-            <v>Neurology</v>
-          </cell>
-          <cell r="B3" t="str">
-            <v>D002</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>Dr. Mehta</v>
-          </cell>
-          <cell r="E3">
-            <v>40</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>Orthopedics</v>
-          </cell>
-          <cell r="B4" t="str">
-            <v>D003</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>Dr. Kumar</v>
-          </cell>
-          <cell r="E4">
-            <v>60</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>Pediatrics</v>
-          </cell>
-          <cell r="B5" t="str">
-            <v>D004</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>Dr. Sharma</v>
-          </cell>
-          <cell r="E5">
-            <v>35</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>Emergency</v>
-          </cell>
-          <cell r="B6" t="str">
-            <v>D005</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>Dr. Reddy</v>
-          </cell>
-          <cell r="E6">
-            <v>70</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Praveen Tirumani" refreshedDate="46145.476931944446" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="30" xr:uid="{45B2C812-339F-428F-8ACC-78175B2DC9CC}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:K31" sheet="Patient_records" r:id="rId2"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Patient ID" numFmtId="0">
+      <sharedItems count="30">
+        <s v="A10001"/>
+        <s v="A10002"/>
+        <s v="A10003"/>
+        <s v="A10004"/>
+        <s v="A10005"/>
+        <s v="A10006"/>
+        <s v="A10007"/>
+        <s v="A10008"/>
+        <s v="A10009"/>
+        <s v="A10010"/>
+        <s v="A10011"/>
+        <s v="A10012"/>
+        <s v="A10013"/>
+        <s v="A10014"/>
+        <s v="A10015"/>
+        <s v="A10016"/>
+        <s v="A10017"/>
+        <s v="A10018"/>
+        <s v="A10019"/>
+        <s v="A10020"/>
+        <s v="A10021"/>
+        <s v="A10022"/>
+        <s v="A10023"/>
+        <s v="A10024"/>
+        <s v="A10025"/>
+        <s v="A10026"/>
+        <s v="A10027"/>
+        <s v="A10028"/>
+        <s v="A10029"/>
+        <s v="A10030"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Name " numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Age" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="45"/>
+    </cacheField>
+    <cacheField name="Gender" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="City" numFmtId="0">
+      <sharedItems count="19">
+        <s v="Hyderabad"/>
+        <s v="Gudivada"/>
+        <s v="Begumpet"/>
+        <s v="Amaravathi"/>
+        <s v="Godavari"/>
+        <s v="Konaseema"/>
+        <s v="Malakpet"/>
+        <s v="Kondaput"/>
+        <s v="Hafeezpet"/>
+        <s v="High tech city"/>
+        <s v="Kondapur"/>
+        <s v="Nandigama"/>
+        <s v="Singareni"/>
+        <s v="Rajkot"/>
+        <s v="Bengalore"/>
+        <s v="Vizag"/>
+        <s v="Petrorius"/>
+        <s v="Nalgonda"/>
+        <s v="Chennai"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Appointment Date" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-30T00:00:00" maxDate="2026-05-30T00:00:00" count="30">
+        <d v="2026-04-30T00:00:00"/>
+        <d v="2026-05-01T00:00:00"/>
+        <d v="2026-05-02T00:00:00"/>
+        <d v="2026-05-03T00:00:00"/>
+        <d v="2026-05-04T00:00:00"/>
+        <d v="2026-05-05T00:00:00"/>
+        <d v="2026-05-06T00:00:00"/>
+        <d v="2026-05-07T00:00:00"/>
+        <d v="2026-05-08T00:00:00"/>
+        <d v="2026-05-09T00:00:00"/>
+        <d v="2026-05-10T00:00:00"/>
+        <d v="2026-05-11T00:00:00"/>
+        <d v="2026-05-12T00:00:00"/>
+        <d v="2026-05-13T00:00:00"/>
+        <d v="2026-05-14T00:00:00"/>
+        <d v="2026-05-15T00:00:00"/>
+        <d v="2026-05-16T00:00:00"/>
+        <d v="2026-05-17T00:00:00"/>
+        <d v="2026-05-18T00:00:00"/>
+        <d v="2026-05-19T00:00:00"/>
+        <d v="2026-05-20T00:00:00"/>
+        <d v="2026-05-21T00:00:00"/>
+        <d v="2026-05-22T00:00:00"/>
+        <d v="2026-05-23T00:00:00"/>
+        <d v="2026-05-24T00:00:00"/>
+        <d v="2026-05-25T00:00:00"/>
+        <d v="2026-05-26T00:00:00"/>
+        <d v="2026-05-27T00:00:00"/>
+        <d v="2026-05-28T00:00:00"/>
+        <d v="2026-05-29T00:00:00"/>
+      </sharedItems>
+      <fieldGroup par="11"/>
+    </cacheField>
+    <cacheField name="Dapartment Name" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Cardiology"/>
+        <s v="Emergency"/>
+        <s v="Neurology"/>
+        <s v="Pediatrics"/>
+        <s v="Orthopedics"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Showed Up" numFmtId="0">
+      <sharedItems count="2">
+        <s v="Yes"/>
+        <s v="No"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Department ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Head Doctor" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Bed Capacity" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="35" maxValue="70"/>
+    </cacheField>
+    <cacheField name="Months (Appointment Date)" numFmtId="0" databaseField="0">
+      <fieldGroup base="5">
+        <rangePr groupBy="months" startDate="2026-04-30T00:00:00" endDate="2026-05-30T00:00:00"/>
+        <groupItems count="14">
+          <s v="&lt;30-04-2026"/>
+          <s v="Jan"/>
+          <s v="Feb"/>
+          <s v="Mar"/>
+          <s v="Apr"/>
+          <s v="May"/>
+          <s v="Jun"/>
+          <s v="Jul"/>
+          <s v="Aug"/>
+          <s v="Sep"/>
+          <s v="Oct"/>
+          <s v="Nov"/>
+          <s v="Dec"/>
+          <s v="&gt;30-05-2026"/>
+        </groupItems>
+      </fieldGroup>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Praveen Tirumani" refreshedDate="46145.477733564818" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="30" xr:uid="{49747DB3-F6CB-460E-B16F-1BC4E077B54A}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:L31" sheet="Patient_records" r:id="rId2"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Patient ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Name " numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Age" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="18" maxValue="45"/>
+    </cacheField>
+    <cacheField name="Gender" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="City" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Appointment Date" numFmtId="14">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-04-30T00:00:00" maxDate="2026-05-30T00:00:00"/>
+    </cacheField>
+    <cacheField name="Dapartment Name" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Cardiology"/>
+        <s v="Emergency"/>
+        <s v="Neurology"/>
+        <s v="Pediatrics"/>
+        <s v="Orthopedics"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Showed Up" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Department ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Head Doctor" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Bed Capacity" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="35" maxValue="70"/>
+    </cacheField>
+    <cacheField name="Senior category" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="30">
+  <r>
+    <x v="0"/>
+    <s v="Praveen"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <s v="Dhanush"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <s v="Harpreet"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <s v="Sekhar"/>
+    <n v="19"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <s v="Rangayya"/>
+    <n v="20"/>
+    <s v="Male"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <s v="Rangamma"/>
+    <n v="18"/>
+    <s v="Female"/>
+    <x v="1"/>
+    <x v="5"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <s v="Mogalayya"/>
+    <n v="25"/>
+    <s v="Male"/>
+    <x v="2"/>
+    <x v="6"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <s v="Jangayya"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <x v="3"/>
+    <x v="7"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <s v="Madhu"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="4"/>
+    <x v="8"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <s v="Rudra"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="5"/>
+    <x v="9"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="10"/>
+    <s v="Mehar"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <x v="6"/>
+    <x v="10"/>
+    <x v="3"/>
+    <x v="0"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="11"/>
+    <s v="mohan"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="7"/>
+    <x v="11"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="12"/>
+    <s v="Radhika"/>
+    <n v="22"/>
+    <s v="Female"/>
+    <x v="8"/>
+    <x v="12"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="13"/>
+    <s v="Mounika"/>
+    <n v="30"/>
+    <s v="Female"/>
+    <x v="9"/>
+    <x v="13"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="14"/>
+    <s v="Meghana"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="10"/>
+    <x v="14"/>
+    <x v="0"/>
+    <x v="1"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="15"/>
+    <s v="Nagalaxmi"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="11"/>
+    <x v="15"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="16"/>
+    <s v="Manoj"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <x v="11"/>
+    <x v="16"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="17"/>
+    <s v="Rekha"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <x v="10"/>
+    <x v="17"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="18"/>
+    <s v="Happie"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <x v="6"/>
+    <x v="18"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="19"/>
+    <s v="Nagarjuna"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <x v="12"/>
+    <x v="19"/>
+    <x v="0"/>
+    <x v="1"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="20"/>
+    <s v="Sikhar"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <x v="13"/>
+    <x v="20"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="21"/>
+    <s v="Dhawan"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <x v="14"/>
+    <x v="21"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="22"/>
+    <s v="Neelambari"/>
+    <n v="34"/>
+    <s v="Female"/>
+    <x v="0"/>
+    <x v="22"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+  <r>
+    <x v="23"/>
+    <s v="Aravind"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="0"/>
+    <x v="23"/>
+    <x v="2"/>
+    <x v="1"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="24"/>
+    <s v="Meghana"/>
+    <n v="24"/>
+    <s v="Female"/>
+    <x v="0"/>
+    <x v="24"/>
+    <x v="3"/>
+    <x v="1"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+  </r>
+  <r>
+    <x v="25"/>
+    <s v="Simha"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="4"/>
+    <x v="25"/>
+    <x v="4"/>
+    <x v="0"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+  </r>
+  <r>
+    <x v="26"/>
+    <s v="Reddy"/>
+    <n v="23"/>
+    <s v="Male"/>
+    <x v="15"/>
+    <x v="26"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="27"/>
+    <s v="Klassen"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <x v="16"/>
+    <x v="27"/>
+    <x v="2"/>
+    <x v="0"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+  </r>
+  <r>
+    <x v="28"/>
+    <s v="Mouna"/>
+    <n v="28"/>
+    <s v="Female"/>
+    <x v="17"/>
+    <x v="28"/>
+    <x v="0"/>
+    <x v="0"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+  </r>
+  <r>
+    <x v="29"/>
+    <s v="Dinesh"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <x v="18"/>
+    <x v="29"/>
+    <x v="1"/>
+    <x v="0"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="30">
+  <r>
+    <s v="A10001"/>
+    <s v="Praveen"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-04-30T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10002"/>
+    <s v="Dhanush"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-01T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10003"/>
+    <s v="Harpreet"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-02T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10004"/>
+    <s v="Sekhar"/>
+    <n v="19"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-03T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10005"/>
+    <s v="Rangayya"/>
+    <n v="20"/>
+    <s v="Male"/>
+    <s v="Gudivada"/>
+    <d v="2026-05-04T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10006"/>
+    <s v="Rangamma"/>
+    <n v="18"/>
+    <s v="Female"/>
+    <s v="Gudivada"/>
+    <d v="2026-05-05T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10007"/>
+    <s v="Mogalayya"/>
+    <n v="25"/>
+    <s v="Male"/>
+    <s v="Begumpet"/>
+    <d v="2026-05-06T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10008"/>
+    <s v="Jangayya"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <s v="Amaravathi"/>
+    <d v="2026-05-07T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10009"/>
+    <s v="Madhu"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Godavari"/>
+    <d v="2026-05-08T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10010"/>
+    <s v="Rudra"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Konaseema"/>
+    <d v="2026-05-09T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10011"/>
+    <s v="Mehar"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <s v="Malakpet"/>
+    <d v="2026-05-10T00:00:00"/>
+    <x v="3"/>
+    <s v="Yes"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10012"/>
+    <s v="mohan"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Kondaput"/>
+    <d v="2026-05-11T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10013"/>
+    <s v="Radhika"/>
+    <n v="22"/>
+    <s v="Female"/>
+    <s v="Hafeezpet"/>
+    <d v="2026-05-12T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10014"/>
+    <s v="Mounika"/>
+    <n v="30"/>
+    <s v="Female"/>
+    <s v="High tech city"/>
+    <d v="2026-05-13T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10015"/>
+    <s v="Meghana"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Kondapur"/>
+    <d v="2026-05-14T00:00:00"/>
+    <x v="0"/>
+    <s v="No"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10016"/>
+    <s v="Nagalaxmi"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Nandigama"/>
+    <d v="2026-05-15T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10017"/>
+    <s v="Manoj"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <s v="Nandigama"/>
+    <d v="2026-05-16T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10018"/>
+    <s v="Rekha"/>
+    <n v="29"/>
+    <s v="Female"/>
+    <s v="Kondapur"/>
+    <d v="2026-05-17T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10019"/>
+    <s v="Happie"/>
+    <n v="20"/>
+    <s v="Female"/>
+    <s v="Malakpet"/>
+    <d v="2026-05-18T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10020"/>
+    <s v="Nagarjuna"/>
+    <n v="29"/>
+    <s v="Male"/>
+    <s v="Singareni"/>
+    <d v="2026-05-19T00:00:00"/>
+    <x v="0"/>
+    <s v="No"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10021"/>
+    <s v="Sikhar"/>
+    <n v="28"/>
+    <s v="Male"/>
+    <s v="Rajkot"/>
+    <d v="2026-05-20T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10022"/>
+    <s v="Dhawan"/>
+    <n v="45"/>
+    <s v="Male"/>
+    <s v="Bengalore"/>
+    <d v="2026-05-21T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10023"/>
+    <s v="Neelambari"/>
+    <n v="34"/>
+    <s v="Female"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-22T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10024"/>
+    <s v="Aravind"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-23T00:00:00"/>
+    <x v="2"/>
+    <s v="No"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10025"/>
+    <s v="Meghana"/>
+    <n v="24"/>
+    <s v="Female"/>
+    <s v="Hyderabad"/>
+    <d v="2026-05-24T00:00:00"/>
+    <x v="3"/>
+    <s v="No"/>
+    <s v="D004"/>
+    <s v="Dr. Sharma"/>
+    <n v="35"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10026"/>
+    <s v="Simha"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Godavari"/>
+    <d v="2026-05-25T00:00:00"/>
+    <x v="4"/>
+    <s v="Yes"/>
+    <s v="D003"/>
+    <s v="Dr. Kumar"/>
+    <n v="60"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10027"/>
+    <s v="Reddy"/>
+    <n v="23"/>
+    <s v="Male"/>
+    <s v="Vizag"/>
+    <d v="2026-05-26T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10028"/>
+    <s v="Klassen"/>
+    <n v="34"/>
+    <s v="Male"/>
+    <s v="Petrorius"/>
+    <d v="2026-05-27T00:00:00"/>
+    <x v="2"/>
+    <s v="Yes"/>
+    <s v="D002"/>
+    <s v="Dr. Mehta"/>
+    <n v="40"/>
+    <s v="Senior"/>
+  </r>
+  <r>
+    <s v="A10029"/>
+    <s v="Mouna"/>
+    <n v="28"/>
+    <s v="Female"/>
+    <s v="Nalgonda"/>
+    <d v="2026-05-28T00:00:00"/>
+    <x v="0"/>
+    <s v="Yes"/>
+    <s v="D001"/>
+    <s v="Dr. Rao"/>
+    <n v="50"/>
+    <s v="Normal"/>
+  </r>
+  <r>
+    <s v="A10030"/>
+    <s v="Dinesh"/>
+    <n v="22"/>
+    <s v="Male"/>
+    <s v="Chennai"/>
+    <d v="2026-05-29T00:00:00"/>
+    <x v="1"/>
+    <s v="Yes"/>
+    <s v="D005"/>
+    <s v="Dr. Reddy"/>
+    <n v="70"/>
+    <s v="Normal"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59BB44AF-A5BC-4037-BA48-5B9F8ECA1576}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="O4:T25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="20">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="18"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="15"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="20">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="6" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72018C71-081E-430C-9EFB-434E0137579D}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="A17:B23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Age" fld="2" subtotal="average" baseField="6" baseItem="2" numFmtId="164"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="0">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D282C46E-B6AC-4BD1-A38E-4B2CD3E63F3E}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J17:K21" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="12">
+    <pivotField axis="axisPage" dataField="1" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" measureFilter="1" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="1"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="1">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <filters count="1">
+    <filter fld="6" type="count" evalOrder="-1" id="1" iMeasureFld="0">
+      <autoFilter ref="A1">
+        <filterColumn colId="0">
+          <top10 val="3" filterVal="3"/>
+        </filterColumn>
+      </autoFilter>
+    </filter>
+  </filters>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5BC9A949-698A-4F91-A460-B4E7FA01B804}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J4:L11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="7" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" showDataAs="percentOfTotal" baseField="6" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8360A506-32EC-4E07-8FAB-7878DFF8E6A5}" name="PivotTable9" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="city">
+  <location ref="A29:D50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="20">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="14"/>
+        <item x="18"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="16"/>
+        <item x="13"/>
+        <item x="12"/>
+        <item x="15"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="20">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="4">
+    <format dxfId="2">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="18">
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="12"/>
+            <x v="13"/>
+            <x v="14"/>
+            <x v="15"/>
+            <x v="16"/>
+            <x v="17"/>
+            <x v="18"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3E335D19-276A-4D6A-8CED-9797D932BF7B}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Months">
+  <location ref="E17:F20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="11"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="4">
+    <format dxfId="6">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="8">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="11" count="1">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BBE503ED-5965-48DF-869B-897BBB276DDD}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="A4:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{21A999CC-767A-459F-BDBF-E65A267B5DFF}" name="PivotTable11" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="J29:K35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Senior category" fld="11" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7A8372AE-A8EB-4B05-AA13-AC82AD570621}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Departments">
+  <location ref="E4:G11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="31">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="7" count="1" selected="0">
+              <x v="1"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="7"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Patient ID" fld="0" subtotal="count" showDataAs="percentOfTotal" baseField="6" baseItem="0" numFmtId="10"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -797,6 +3257,1066 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1CE93FF-A88A-47E3-B89B-D6BE459E2132}">
+  <dimension ref="A4:T50"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" customWidth="1"/>
+    <col min="11" max="11" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="O4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="P4" s="9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>9</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="K5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" t="s">
+        <v>0</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="P5" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>1</v>
+      </c>
+      <c r="R5" t="s">
+        <v>11</v>
+      </c>
+      <c r="S5" t="s">
+        <v>18</v>
+      </c>
+      <c r="T5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="10">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K6" s="10">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L6" s="10">
+        <v>0.23333333333333334</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="P6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K7" s="10">
+        <v>0</v>
+      </c>
+      <c r="L7" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="L8" s="10">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="10">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="10">
+        <v>0</v>
+      </c>
+      <c r="L9" s="10">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10">
+        <v>30</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="10">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K10" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="10">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="E11" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F11" s="10">
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0.73333333333333328</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="K11" s="10">
+        <v>0.26666666666666666</v>
+      </c>
+      <c r="L11" s="10">
+        <v>0.73333333333333328</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
+      <c r="S11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O12" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="P12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O13" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14">
+        <v>2</v>
+      </c>
+      <c r="R14">
+        <v>2</v>
+      </c>
+      <c r="T14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="J15" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="K15" t="s">
+        <v>126</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O16" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16">
+        <v>1</v>
+      </c>
+      <c r="T16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" t="s">
+        <v>121</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="K17" t="s">
+        <v>121</v>
+      </c>
+      <c r="O17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="S17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A18" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="3">
+        <v>28.666666666666668</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="F18" s="7">
+        <v>29</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K18" s="7">
+        <v>9</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="S18">
+        <v>1</v>
+      </c>
+      <c r="T18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" s="3">
+        <v>24</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="7">
+        <v>1</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K19" s="7">
+        <v>8</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="P19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A20" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="3">
+        <v>27.25</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="7">
+        <v>30</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K20" s="7">
+        <v>5</v>
+      </c>
+      <c r="O20" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q20">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="3">
+        <v>27</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="K21" s="7">
+        <v>22</v>
+      </c>
+      <c r="O21" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="R21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="3">
+        <v>25.25</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="R22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" s="3">
+        <v>26.833333333333332</v>
+      </c>
+      <c r="O23" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="P23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O24" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="P24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="O25" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="P25">
+        <v>9</v>
+      </c>
+      <c r="Q25">
+        <v>5</v>
+      </c>
+      <c r="R25">
+        <v>8</v>
+      </c>
+      <c r="S25">
+        <v>4</v>
+      </c>
+      <c r="T25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="J29" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="K29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B30" t="s">
+        <v>22</v>
+      </c>
+      <c r="C30" t="s">
+        <v>0</v>
+      </c>
+      <c r="D30" t="s">
+        <v>116</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K30">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A31" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7">
+        <v>1</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A32" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7">
+        <v>1</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K32">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7">
+        <v>1</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7">
+        <v>1</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K34">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7">
+        <v>2</v>
+      </c>
+      <c r="D35" s="7">
+        <v>2</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="K35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7">
+        <v>1</v>
+      </c>
+      <c r="D38" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B39" s="7">
+        <v>4</v>
+      </c>
+      <c r="C39" s="7">
+        <v>3</v>
+      </c>
+      <c r="D39" s="7">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7">
+        <v>1</v>
+      </c>
+      <c r="D40" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="7">
+        <v>2</v>
+      </c>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7">
+        <v>2</v>
+      </c>
+      <c r="D43" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="7">
+        <v>1</v>
+      </c>
+      <c r="C45" s="7">
+        <v>1</v>
+      </c>
+      <c r="D45" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7">
+        <v>1</v>
+      </c>
+      <c r="D46" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7">
+        <v>1</v>
+      </c>
+      <c r="D47" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" s="7">
+        <v>1</v>
+      </c>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7">
+        <v>1</v>
+      </c>
+      <c r="D49" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" s="7">
+        <v>8</v>
+      </c>
+      <c r="C50" s="7">
+        <v>22</v>
+      </c>
+      <c r="D50" s="7">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{893ED410-0D4C-4F44-AE6B-6CE91E33D4B8}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" customWidth="1"/>
+    <col min="7" max="7" width="33.88671875" customWidth="1"/>
+    <col min="8" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="9" width="16.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="4">
+        <v>50</v>
+      </c>
+      <c r="F2">
+        <f>COUNTIF(Patient_records!$J$2:$J$31,Department_info!D2)</f>
+        <v>9</v>
+      </c>
+      <c r="G2" s="3">
+        <f>AVERAGEIF(Patient_records!$G$2:$G$31,Department_info!A2,Patient_records!$C$2:$C$31)</f>
+        <v>28.666666666666668</v>
+      </c>
+      <c r="H2" s="3">
+        <f>COUNTIF(Patient_records!$G$2:$G$31,Department_info!A2) / Department_info!E2</f>
+        <v>0.18</v>
+      </c>
+      <c r="I2" t="str">
+        <f>IF(H2&gt;0.8,"Over Capacity","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="4">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E3" s="4">
+        <v>40</v>
+      </c>
+      <c r="F3">
+        <f>COUNTIF(Patient_records!$J$2:$J$31,Department_info!D3)</f>
+        <v>8</v>
+      </c>
+      <c r="G3" s="3">
+        <f>AVERAGEIF(Patient_records!$G$2:$G$31,Department_info!A3,Patient_records!$C$2:$C$31)</f>
+        <v>27.25</v>
+      </c>
+      <c r="H3" s="3">
+        <f>COUNTIF(Patient_records!$G$2:$G$31,Department_info!A3) / Department_info!E3</f>
+        <v>0.2</v>
+      </c>
+      <c r="I3" t="str">
+        <f>IF(H3&gt;0.8,"Over Capacity","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" s="4">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <f>COUNTIF(Patient_records!$J$2:$J$31,Department_info!D4)</f>
+        <v>4</v>
+      </c>
+      <c r="G4" s="3">
+        <f>AVERAGEIF(Patient_records!$G$2:$G$31,Department_info!A4,Patient_records!$C$2:$C$31)</f>
+        <v>27</v>
+      </c>
+      <c r="H4" s="3">
+        <f>COUNTIF(Patient_records!$G$2:$G$31,Department_info!A4) / Department_info!E4</f>
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="I4" t="str">
+        <f>IF(H4&gt;0.8,"Over Capacity","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E5" s="4">
+        <v>35</v>
+      </c>
+      <c r="F5">
+        <f>COUNTIF(Patient_records!$J$2:$J$31,Department_info!D5)</f>
+        <v>4</v>
+      </c>
+      <c r="G5" s="3">
+        <f>AVERAGEIF(Patient_records!$G$2:$G$31,Department_info!A5,Patient_records!$C$2:$C$31)</f>
+        <v>25.25</v>
+      </c>
+      <c r="H5" s="3">
+        <f>COUNTIF(Patient_records!$G$2:$G$31,Department_info!A5) / Department_info!E5</f>
+        <v>0.11428571428571428</v>
+      </c>
+      <c r="I5" t="str">
+        <f>IF(H5&gt;0.8,"Over Capacity","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="4">
+        <v>70</v>
+      </c>
+      <c r="F6">
+        <f>COUNTIF(Patient_records!$J$2:$J$31,Department_info!D6)</f>
+        <v>5</v>
+      </c>
+      <c r="G6" s="3">
+        <f>AVERAGEIF(Patient_records!$G$2:$G$31,Department_info!A6,Patient_records!$C$2:$C$31)</f>
+        <v>24</v>
+      </c>
+      <c r="H6" s="3">
+        <f>COUNTIF(Patient_records!$G$2:$G$31,Department_info!A6) / Department_info!E6</f>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="I6" t="str">
+        <f>IF(H6&gt;0.8,"Over Capacity","Normal")</f>
+        <v>Normal</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32083944-5797-4D68-90B6-E0A040CDCA6A}">
   <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -879,19 +4399,19 @@
         <v>0</v>
       </c>
       <c r="I2" t="str">
-        <f>VLOOKUP(G2,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G2,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J2" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G2,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G2,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K2">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G2,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G2,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L2" t="str">
-        <f>IF(C2&gt;30,"Senior","Normal")</f>
+        <f t="shared" ref="L2:L31" si="0">IF(C2&gt;30,"Senior","Normal")</f>
         <v>Normal</v>
       </c>
     </row>
@@ -921,19 +4441,19 @@
         <v>0</v>
       </c>
       <c r="I3" t="str">
-        <f>VLOOKUP(G3,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G3,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D005</v>
       </c>
       <c r="J3" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G3,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G3,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Reddy</v>
       </c>
       <c r="K3">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G3,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G3,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
       <c r="L3" t="str">
-        <f>IF(C3&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -963,19 +4483,19 @@
         <v>22</v>
       </c>
       <c r="I4" t="str">
-        <f>VLOOKUP(G4,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G4,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J4" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G4,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G4,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K4">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G4,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G4,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L4" t="str">
-        <f>IF(C4&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1005,19 +4525,19 @@
         <v>22</v>
       </c>
       <c r="I5" t="str">
-        <f>VLOOKUP(G5,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G5,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D004</v>
       </c>
       <c r="J5" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G5,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G5,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Sharma</v>
       </c>
       <c r="K5">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G5,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G5,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
       <c r="L5" t="str">
-        <f>IF(C5&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1047,19 +4567,19 @@
         <v>0</v>
       </c>
       <c r="I6" t="str">
-        <f>VLOOKUP(G6,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G6,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D003</v>
       </c>
       <c r="J6" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G6,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G6,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Kumar</v>
       </c>
       <c r="K6">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G6,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G6,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
       <c r="L6" t="str">
-        <f>IF(C6&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1089,19 +4609,19 @@
         <v>0</v>
       </c>
       <c r="I7" t="str">
-        <f>VLOOKUP(G7,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G7,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J7" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G7,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G7,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K7">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G7,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G7,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L7" t="str">
-        <f>IF(C7&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1131,19 +4651,19 @@
         <v>0</v>
       </c>
       <c r="I8" t="str">
-        <f>VLOOKUP(G8,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G8,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J8" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G8,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G8,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K8">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G8,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G8,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L8" t="str">
-        <f>IF(C8&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1173,19 +4693,19 @@
         <v>0</v>
       </c>
       <c r="I9" t="str">
-        <f>VLOOKUP(G9,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G9,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J9" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G9,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G9,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K9">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G9,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G9,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L9" t="str">
-        <f>IF(C9&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -1215,19 +4735,19 @@
         <v>0</v>
       </c>
       <c r="I10" t="str">
-        <f>VLOOKUP(G10,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G10,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D005</v>
       </c>
       <c r="J10" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G10,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G10,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Reddy</v>
       </c>
       <c r="K10">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G10,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G10,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
       <c r="L10" t="str">
-        <f>IF(C10&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1257,19 +4777,19 @@
         <v>0</v>
       </c>
       <c r="I11" t="str">
-        <f>VLOOKUP(G11,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G11,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J11" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G11,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G11,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K11">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G11,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G11,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L11" t="str">
-        <f>IF(C11&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1299,19 +4819,19 @@
         <v>0</v>
       </c>
       <c r="I12" t="str">
-        <f>VLOOKUP(G12,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G12,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D004</v>
       </c>
       <c r="J12" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G12,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G12,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Sharma</v>
       </c>
       <c r="K12">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G12,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G12,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
       <c r="L12" t="str">
-        <f>IF(C12&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1341,19 +4861,19 @@
         <v>0</v>
       </c>
       <c r="I13" t="str">
-        <f>VLOOKUP(G13,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G13,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D003</v>
       </c>
       <c r="J13" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G13,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G13,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Kumar</v>
       </c>
       <c r="K13">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G13,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G13,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
       <c r="L13" t="str">
-        <f>IF(C13&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -1383,19 +4903,19 @@
         <v>0</v>
       </c>
       <c r="I14" t="str">
-        <f>VLOOKUP(G14,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G14,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J14" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G14,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G14,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K14">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G14,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G14,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L14" t="str">
-        <f>IF(C14&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1425,19 +4945,19 @@
         <v>0</v>
       </c>
       <c r="I15" t="str">
-        <f>VLOOKUP(G15,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G15,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J15" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G15,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G15,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K15">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G15,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G15,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L15" t="str">
-        <f>IF(C15&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1467,19 +4987,19 @@
         <v>22</v>
       </c>
       <c r="I16" t="str">
-        <f>VLOOKUP(G16,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G16,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J16" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G16,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G16,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K16">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G16,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G16,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L16" t="str">
-        <f>IF(C16&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1509,19 +5029,19 @@
         <v>0</v>
       </c>
       <c r="I17" t="str">
-        <f>VLOOKUP(G17,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G17,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D005</v>
       </c>
       <c r="J17" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G17,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G17,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Reddy</v>
       </c>
       <c r="K17">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G17,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G17,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
       <c r="L17" t="str">
-        <f>IF(C17&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1551,19 +5071,19 @@
         <v>22</v>
       </c>
       <c r="I18" t="str">
-        <f>VLOOKUP(G18,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G18,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J18" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G18,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G18,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K18">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G18,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G18,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L18" t="str">
-        <f>IF(C18&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1593,19 +5113,19 @@
         <v>22</v>
       </c>
       <c r="I19" t="str">
-        <f>VLOOKUP(G19,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G19,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D004</v>
       </c>
       <c r="J19" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G19,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G19,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Sharma</v>
       </c>
       <c r="K19">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G19,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G19,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
       <c r="L19" t="str">
-        <f>IF(C19&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1635,19 +5155,19 @@
         <v>0</v>
       </c>
       <c r="I20" t="str">
-        <f>VLOOKUP(G20,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G20,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D003</v>
       </c>
       <c r="J20" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G20,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G20,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Kumar</v>
       </c>
       <c r="K20">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G20,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G20,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
       <c r="L20" t="str">
-        <f>IF(C20&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1677,19 +5197,19 @@
         <v>22</v>
       </c>
       <c r="I21" t="str">
-        <f>VLOOKUP(G21,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G21,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J21" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G21,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G21,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K21">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G21,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G21,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L21" t="str">
-        <f>IF(C21&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1719,19 +5239,19 @@
         <v>0</v>
       </c>
       <c r="I22" t="str">
-        <f>VLOOKUP(G22,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G22,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J22" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G22,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G22,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K22">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G22,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G22,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L22" t="str">
-        <f>IF(C22&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1761,19 +5281,19 @@
         <v>0</v>
       </c>
       <c r="I23" t="str">
-        <f>VLOOKUP(G23,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G23,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J23" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G23,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G23,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K23">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G23,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G23,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L23" t="str">
-        <f>IF(C23&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -1803,19 +5323,19 @@
         <v>0</v>
       </c>
       <c r="I24" t="str">
-        <f>VLOOKUP(G24,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G24,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D005</v>
       </c>
       <c r="J24" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G24,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G24,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Reddy</v>
       </c>
       <c r="K24">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G24,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G24,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
       <c r="L24" t="str">
-        <f>IF(C24&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -1845,19 +5365,19 @@
         <v>22</v>
       </c>
       <c r="I25" t="str">
-        <f>VLOOKUP(G25,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G25,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J25" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G25,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G25,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K25">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G25,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G25,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L25" t="str">
-        <f>IF(C25&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1887,19 +5407,19 @@
         <v>22</v>
       </c>
       <c r="I26" t="str">
-        <f>VLOOKUP(G26,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G26,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D004</v>
       </c>
       <c r="J26" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G26,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G26,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Sharma</v>
       </c>
       <c r="K26">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G26,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G26,Department_info!$A$2:$A$6,0))</f>
         <v>35</v>
       </c>
       <c r="L26" t="str">
-        <f>IF(C26&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -1929,19 +5449,19 @@
         <v>0</v>
       </c>
       <c r="I27" t="str">
-        <f>VLOOKUP(G27,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G27,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D003</v>
       </c>
       <c r="J27" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G27,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G27,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Kumar</v>
       </c>
       <c r="K27">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G27,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G27,Department_info!$A$2:$A$6,0))</f>
         <v>60</v>
       </c>
       <c r="L27" t="str">
-        <f>IF(C27&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -1971,19 +5491,19 @@
         <v>0</v>
       </c>
       <c r="I28" t="str">
-        <f>VLOOKUP(G28,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G28,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J28" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G28,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G28,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K28">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G28,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G28,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L28" t="str">
-        <f>IF(C28&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -2013,19 +5533,19 @@
         <v>0</v>
       </c>
       <c r="I29" t="str">
-        <f>VLOOKUP(G29,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G29,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D002</v>
       </c>
       <c r="J29" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G29,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G29,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Mehta</v>
       </c>
       <c r="K29">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G29,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G29,Department_info!$A$2:$A$6,0))</f>
         <v>40</v>
       </c>
       <c r="L29" t="str">
-        <f>IF(C29&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Senior</v>
       </c>
     </row>
@@ -2055,19 +5575,19 @@
         <v>0</v>
       </c>
       <c r="I30" t="str">
-        <f>VLOOKUP(G30,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G30,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D001</v>
       </c>
       <c r="J30" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G30,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G30,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Rao</v>
       </c>
       <c r="K30">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G30,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G30,Department_info!$A$2:$A$6,0))</f>
         <v>50</v>
       </c>
       <c r="L30" t="str">
-        <f>IF(C30&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
@@ -2097,32 +5617,23 @@
         <v>0</v>
       </c>
       <c r="I31" t="str">
-        <f>VLOOKUP(G31,[1]Department_info!$A$2:$B$6,2,FALSE)</f>
+        <f>VLOOKUP(G31,Department_info!$A$2:$B$6,2,FALSE)</f>
         <v>D005</v>
       </c>
       <c r="J31" t="str">
-        <f>INDEX([1]Department_info!$D$2:$D$6,MATCH(Patient_records!G31,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$D$2:$D$6,MATCH(Patient_records!G31,Department_info!$A$2:$A$6,0))</f>
         <v>Dr. Reddy</v>
       </c>
       <c r="K31">
-        <f>INDEX([1]Department_info!$E$2:$E$6,MATCH(Patient_records!G31,[1]Department_info!$A$2:$A$6,0))</f>
+        <f>INDEX(Department_info!$E$2:$E$6,MATCH(Patient_records!G31,Department_info!$A$2:$A$6,0))</f>
         <v>70</v>
       </c>
       <c r="L31" t="str">
-        <f>IF(C31&gt;30,"Senior","Normal")</f>
+        <f t="shared" si="0"/>
         <v>Normal</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D985C4CB-ED47-45C2-9924-BB4AB878FE9D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>